<commit_message>
Alterado Formato de Data aba Inconsistencia
</commit_message>
<xml_diff>
--- a/relatorio_final.xlsx
+++ b/relatorio_final.xlsx
@@ -62,7 +62,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -70,7 +70,6 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1275,7 +1274,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n">
+      <c r="A2" s="3" t="n">
         <v>46063</v>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>